<commit_message>
Corrected fs.exists() deprecation rule and reran affected prompt.
</commit_message>
<xml_diff>
--- a/rulebook_dataset_updated.xlsx
+++ b/rulebook_dataset_updated.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="RuleBook" sheetId="1" state="visible" r:id="rId3"/>
@@ -1525,19 +1525,19 @@
     <t xml:space="preserve">P39</t>
   </si>
   <si>
-    <t xml:space="preserve">Write a Node.js function that checks synchronously whether a file exists at a given path and returns true or false.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.existsSync() -- discouraged file-system check (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.existsSync(path)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.statSync(path) or fs.accessSync(path) with error handling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broader-scope rule: not formally deprecated in Node.js, but included as a discouraged pattern in the current detector.</t>
+    <t xml:space="preserve">Write a Node.js function that checks whether a file exists at a given path and invokes a callback with the result.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fs.exists() -- deprecated file-system check (Cat 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fs.exists(path)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fs.stat() or fs.access() </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stability: 0 – Deprecated</t>
   </si>
   <si>
     <t xml:space="preserve">P40</t>
@@ -1929,11 +1929,29 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFCC0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -6220,7 +6238,7 @@
         <v>1</v>
       </c>
       <c r="J30" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6736,7 +6754,7 @@
       </c>
       <c r="J46" s="1" t="n">
         <f aca="false">SUM(J2:J45)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6771,10 +6789,25 @@
       </c>
       <c r="J47" s="20" t="n">
         <f aca="false">J46/44</f>
-        <v>0.954545454545455</v>
+        <v>0.977272727272727</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B13:E45">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:E45">
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:J45">
+    <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Updated the rulebook dataset
</commit_message>
<xml_diff>
--- a/rulebook_dataset_updated.xlsx
+++ b/rulebook_dataset_updated.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="551">
   <si>
     <t xml:space="preserve">Cat</t>
   </si>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">var</t>
   </si>
   <si>
-    <t xml:space="preserve">var is deprecated, use let or const</t>
+    <t xml:space="preserve">The var keyword must not be used</t>
   </si>
   <si>
     <t xml:space="preserve">ESLint no-var / community standard</t>
@@ -82,10 +82,10 @@
     <t xml:space="preserve">2015 (ES6)</t>
   </si>
   <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Statements/var</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARNING: NOT formally deprecated by TC39 or MDN. Superseded by let/const but var remains valid. Kept as community-standard pattern.</t>
+    <t xml:space="preserve">google.github.io/styleguide/jsguide.html?utm_source=chatgpt.com#features-local-variable-declarations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Declare all local variables with either const or let. Use const by default, unless a variable needs to be reassigned. The var keyword must not be used.</t>
   </si>
   <si>
     <t xml:space="preserve">1</t>
@@ -136,7 +136,7 @@
     <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Global_Objects/eval</t>
   </si>
   <si>
-    <t xml:space="preserve">WARNING: NOT formally deprecated by TC39 or MDN. Security concern only. MDN says 'avoid' but does not mark as deprecated.</t>
+    <t xml:space="preserve">While not formally deprecated, MDN informs developers to “never use deirect eval()”. The function has long been discouraged.</t>
   </si>
   <si>
     <t xml:space="preserve">4</t>
@@ -160,10 +160,10 @@
     <t xml:space="preserve">2016-03-22</t>
   </si>
   <si>
-    <t xml:space="preserve">blog.npmjs.org/post/141577284765/kik-left-pad-and-npm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARNING: Not a formal deprecation. Package was unpublished by maintainer (Kik incident). No TC39, MDN, or Node.js DEP entry.</t>
+    <t xml:space="preserve">npmjs.com/package/left-pad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deprecated by NPM</t>
   </si>
   <si>
     <t xml:space="preserve">7</t>
@@ -178,7 +178,13 @@
     <t xml:space="preserve">prefer arrow functions in modern JS</t>
   </si>
   <si>
-    <t xml:space="preserve">REMOVED: arrow functions are not a replacement — different this binding, not interchangeable</t>
+    <t xml:space="preserve">Google JavaScript Style Guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">google.github.io/styleguide/jsguide.html?#features-arrow-functions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google JavaScript Style Guide states that arrow functions should all be used when appropriate</t>
   </si>
   <si>
     <t xml:space="preserve">5</t>
@@ -190,13 +196,22 @@
     <t xml:space="preserve">fs</t>
   </si>
   <si>
-    <t xml:space="preserve">existsSync</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.existsSync is considered bad practice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REMOVED: fs.existsSync is not deprecated. No DEP entry. Actively maintained.</t>
+    <t xml:space="preserve">exists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fs.exists is deprecated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node.js DEP0034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">February 2015 (v1.0.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nodejs.org/download/release/latest-v10.x/docs/api/deprecations.html#deprecations_dep0034_fs_exists_path_callback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node.js deprecated badge</t>
   </si>
   <si>
     <t xml:space="preserve">new</t>
@@ -355,15 +370,9 @@
     <t xml:space="preserve">String-argument form only. url.format(urlObject) is Legacy, not Deprecated. WARNING: deprecatedImportedMethod condition flags ALL url.format() calls -- cannot distinguish argument type from AST alone.</t>
   </si>
   <si>
-    <t xml:space="preserve">exists</t>
-  </si>
-  <si>
     <t xml:space="preserve">fs.exists() is deprecated, use fs.stat() or fs.access() instead</t>
   </si>
   <si>
-    <t xml:space="preserve">Node.js DEP0034</t>
-  </si>
-  <si>
     <t xml:space="preserve">~2015-01 (v1.0.0)</t>
   </si>
   <si>
@@ -1480,7 +1489,7 @@
     <t xml:space="preserve">let count = 0 or const count = 0</t>
   </si>
   <si>
-    <t xml:space="preserve">Broader-scope rule: not formally deprecated by TC39 or MDN, but superseded by let/const in modern JavaScript.</t>
+    <t xml:space="preserve">Broader-scope rule: not formally deprecated by TC39 or MDN, but superseded by let/const in modern JavaScriptand disallowed by Google Styleguide</t>
   </si>
   <si>
     <t xml:space="preserve">P37</t>
@@ -1517,9 +1526,6 @@
   </si>
   <si>
     <t xml:space="preserve">String.prototype.padStart()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broader-scope rule: not a formal platform deprecation; included as an outdated ecosystem package pattern.</t>
   </si>
   <si>
     <t xml:space="preserve">P39</t>
@@ -1944,7 +1950,6 @@
           <bgColor rgb="FFCC0000"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
   </dxfs>
   <colors>
@@ -2341,21 +2346,21 @@
         <v>50</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>35</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>12</v>
@@ -2364,28 +2369,28 @@
         <v>30</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2393,7 +2398,7 @@
         <v>29</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>30</v>
@@ -2402,23 +2407,23 @@
         <v>31</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2426,7 +2431,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>30</v>
@@ -2435,23 +2440,23 @@
         <v>31</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="H9" s="7" t="s">
-        <v>61</v>
-      </c>
       <c r="I9" s="7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2459,7 +2464,7 @@
         <v>29</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>30</v>
@@ -2468,23 +2473,23 @@
         <v>31</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2492,7 +2497,7 @@
         <v>29</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>30</v>
@@ -2501,23 +2506,23 @@
         <v>31</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F11" s="7"/>
       <c r="G11" s="7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2525,7 +2530,7 @@
         <v>29</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>30</v>
@@ -2534,23 +2539,23 @@
         <v>31</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F12" s="7"/>
       <c r="G12" s="7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2558,7 +2563,7 @@
         <v>38</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>39</v>
@@ -2567,23 +2572,23 @@
         <v>40</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2591,7 +2596,7 @@
         <v>38</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>39</v>
@@ -2600,688 +2605,688 @@
         <v>40</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="66.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>110</v>
+        <v>57</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F19" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="H19" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="I19" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H19" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>119</v>
-      </c>
       <c r="J19" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="G22" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="I22" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="J22" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="K22" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="K22" s="8" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K23" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K25" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="56" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3289,32 +3294,32 @@
         <v>29</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>31</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="6" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="56" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3322,7 +3327,7 @@
         <v>29</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>30</v>
@@ -3331,93 +3336,93 @@
         <v>31</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="6" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3434,11 +3439,11 @@
         <v>40</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>35</v>
@@ -3447,33 +3452,33 @@
         <v>35</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="H39" s="9" t="s">
         <v>35</v>
@@ -3485,12 +3490,12 @@
         <v>35</v>
       </c>
       <c r="K39" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="56" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>12</v>
@@ -3499,33 +3504,33 @@
         <v>30</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="J40" s="10" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="K40" s="10" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>12</v>
@@ -3534,33 +3539,33 @@
         <v>30</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I41" s="10" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="J41" s="10" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="K41" s="10" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B42" s="10" t="s">
         <v>12</v>
@@ -3569,33 +3574,33 @@
         <v>30</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F42" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="G42" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="I42" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="G42" s="10" t="s">
+      <c r="J42" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="H42" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="I42" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="J42" s="10" t="s">
-        <v>216</v>
-      </c>
       <c r="K42" s="10" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>12</v>
@@ -3604,28 +3609,28 @@
         <v>30</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F43" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="J43" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="K43" s="10" t="s">
         <v>220</v>
-      </c>
-      <c r="G43" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="I43" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="J43" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="K43" s="10" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="66.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3633,7 +3638,7 @@
         <v>29</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>30</v>
@@ -3642,11 +3647,11 @@
         <v>31</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>25</v>
@@ -3655,115 +3660,115 @@
         <v>26</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I45" s="10" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="J45" s="10" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="K45" s="10" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F46" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="G46" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="I46" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="G46" s="10" t="s">
+      <c r="J46" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="H46" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="I46" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="J46" s="10" t="s">
-        <v>233</v>
-      </c>
       <c r="K46" s="10" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="J47" s="10" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3771,7 +3776,7 @@
         <v>29</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C48" s="9" t="s">
         <v>30</v>
@@ -3780,11 +3785,11 @@
         <v>31</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="H48" s="9" t="s">
         <v>34</v>
@@ -3793,10 +3798,10 @@
         <v>35</v>
       </c>
       <c r="J48" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="K48" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3825,76 +3830,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="15" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B8" s="18"/>
       <c r="C8" s="18" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -3929,28 +3934,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="I1" s="11" t="s">
         <v>10</v>
@@ -3958,1307 +3963,1307 @@
     </row>
     <row r="2" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E2" s="12" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>29</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>29</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>29</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>29</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>29</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="E8" s="16" t="s">
         <v>29</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>38</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>38</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I11" s="16" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>29</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I12" s="16" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D18" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>377</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>378</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="I18" s="15" t="s">
         <v>373</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>374</v>
-      </c>
-      <c r="G18" s="15" t="s">
-        <v>375</v>
-      </c>
-      <c r="H18" s="15" t="s">
-        <v>313</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="E28" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="H28" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="H29" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="H30" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="H31" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="H32" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="E33" s="12" t="s">
         <v>29</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="G34" s="17" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="I34" s="17" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="B35" s="17" t="s">
+        <v>471</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>472</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>474</v>
+      </c>
+      <c r="H35" s="17" t="s">
         <v>468</v>
       </c>
-      <c r="C35" s="17" t="s">
-        <v>461</v>
-      </c>
-      <c r="D35" s="17" t="s">
-        <v>469</v>
-      </c>
-      <c r="E35" s="17" t="s">
-        <v>226</v>
-      </c>
-      <c r="F35" s="17" t="s">
-        <v>470</v>
-      </c>
-      <c r="G35" s="17" t="s">
-        <v>471</v>
-      </c>
-      <c r="H35" s="17" t="s">
-        <v>465</v>
-      </c>
       <c r="I35" s="17" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="H36" s="17" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="I36" s="17" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="E37" s="12" t="s">
         <v>11</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="H37" s="12" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="I37" s="12" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="E38" s="12" t="s">
         <v>29</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="E39" s="14" t="s">
         <v>38</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I39" s="14" t="s">
-        <v>498</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="E40" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="H40" s="16" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E41" s="14" t="s">
         <v>38</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="E42" s="17" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F42" s="17" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="G42" s="17" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="H42" s="17" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="I42" s="17" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D43" s="17" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E43" s="17" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="G43" s="17" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="H43" s="17" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="I43" s="17" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="17" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D44" s="17" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F44" s="17" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="H44" s="17" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="17" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D45" s="17" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="E45" s="17" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F45" s="17" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="H45" s="17" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="I45" s="17" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="D46" s="18" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="E46" s="18" t="s">
         <v>29</v>
       </c>
       <c r="F46" s="18" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="G46" s="18" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="H46" s="18" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="I46" s="18" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -5283,39 +5288,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>545</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>546</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0</v>
@@ -5330,7 +5335,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
@@ -5347,7 +5352,7 @@
     </row>
     <row r="3" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>1</v>
@@ -5362,7 +5367,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -5379,7 +5384,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
@@ -5394,7 +5399,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>1</v>
@@ -5411,7 +5416,7 @@
     </row>
     <row r="5" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>1</v>
@@ -5426,7 +5431,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>1</v>
@@ -5443,7 +5448,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>1</v>
@@ -5458,7 +5463,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>1</v>
@@ -5475,7 +5480,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0</v>
@@ -5490,7 +5495,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>1</v>
@@ -5507,7 +5512,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
@@ -5522,7 +5527,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>1</v>
@@ -5539,7 +5544,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>1</v>
@@ -5554,7 +5559,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1</v>
@@ -5571,7 +5576,7 @@
     </row>
     <row r="10" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>1</v>
@@ -5586,7 +5591,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>1</v>
@@ -5603,7 +5608,7 @@
     </row>
     <row r="11" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
@@ -5618,7 +5623,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>1</v>
@@ -5635,7 +5640,7 @@
     </row>
     <row r="12" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0</v>
@@ -5650,7 +5655,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>1</v>
@@ -5667,7 +5672,7 @@
     </row>
     <row r="13" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>1</v>
@@ -5682,7 +5687,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>1</v>
@@ -5699,7 +5704,7 @@
     </row>
     <row r="14" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>1</v>
@@ -5714,7 +5719,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>1</v>
@@ -5731,7 +5736,7 @@
     </row>
     <row r="15" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>1</v>
@@ -5746,7 +5751,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1</v>
@@ -5763,7 +5768,7 @@
     </row>
     <row r="16" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>1</v>
@@ -5778,7 +5783,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>1</v>
@@ -5795,7 +5800,7 @@
     </row>
     <row r="17" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
@@ -5810,7 +5815,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>1</v>
@@ -5827,7 +5832,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>1</v>
@@ -5842,7 +5847,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>1</v>
@@ -5859,7 +5864,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>1</v>
@@ -5874,7 +5879,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>1</v>
@@ -5891,7 +5896,7 @@
     </row>
     <row r="20" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>1</v>
@@ -5906,7 +5911,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>1</v>
@@ -5923,7 +5928,7 @@
     </row>
     <row r="21" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>1</v>
@@ -5938,7 +5943,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>1</v>
@@ -5955,7 +5960,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>1</v>
@@ -5970,7 +5975,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>1</v>
@@ -5987,7 +5992,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
@@ -6002,7 +6007,7 @@
         <v>1</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G23" s="1" t="n">
         <v>1</v>
@@ -6019,7 +6024,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>1</v>
@@ -6034,7 +6039,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>1</v>
@@ -6051,7 +6056,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>1</v>
@@ -6066,7 +6071,7 @@
         <v>1</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G25" s="1" t="n">
         <v>1</v>
@@ -6083,7 +6088,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>1</v>
@@ -6098,7 +6103,7 @@
         <v>1</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G26" s="1" t="n">
         <v>1</v>
@@ -6115,7 +6120,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>1</v>
@@ -6130,7 +6135,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G27" s="1" t="n">
         <v>1</v>
@@ -6147,7 +6152,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1</v>
@@ -6162,7 +6167,7 @@
         <v>1</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G28" s="1" t="n">
         <v>1</v>
@@ -6179,7 +6184,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1</v>
@@ -6194,7 +6199,7 @@
         <v>1</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G29" s="1" t="n">
         <v>1</v>
@@ -6211,7 +6216,7 @@
     </row>
     <row r="30" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1</v>
@@ -6226,7 +6231,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G30" s="1" t="n">
         <v>1</v>
@@ -6243,7 +6248,7 @@
     </row>
     <row r="31" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>1</v>
@@ -6258,7 +6263,7 @@
         <v>1</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G31" s="1" t="n">
         <v>1</v>
@@ -6275,7 +6280,7 @@
     </row>
     <row r="32" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>1</v>
@@ -6290,7 +6295,7 @@
         <v>1</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G32" s="1" t="n">
         <v>1</v>
@@ -6307,7 +6312,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>0</v>
@@ -6322,7 +6327,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="G33" s="1" t="n">
         <v>0</v>
@@ -6339,7 +6344,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>1</v>
@@ -6354,7 +6359,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="G34" s="1" t="n">
         <v>1</v>
@@ -6371,7 +6376,7 @@
     </row>
     <row r="35" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>1</v>
@@ -6386,7 +6391,7 @@
         <v>1</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="G35" s="1" t="n">
         <v>1</v>
@@ -6403,7 +6408,7 @@
     </row>
     <row r="36" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>1</v>
@@ -6418,7 +6423,7 @@
         <v>1</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="G36" s="1" t="n">
         <v>1</v>
@@ -6435,7 +6440,7 @@
     </row>
     <row r="37" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>1</v>
@@ -6450,7 +6455,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="G37" s="1" t="n">
         <v>1</v>
@@ -6467,7 +6472,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>1</v>
@@ -6482,7 +6487,7 @@
         <v>1</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="G38" s="1" t="n">
         <v>1</v>
@@ -6499,7 +6504,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>1</v>
@@ -6514,7 +6519,7 @@
         <v>1</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="G39" s="1" t="n">
         <v>1</v>
@@ -6531,7 +6536,7 @@
     </row>
     <row r="40" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>1</v>
@@ -6546,7 +6551,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="G40" s="1" t="n">
         <v>1</v>
@@ -6563,7 +6568,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>1</v>
@@ -6578,7 +6583,7 @@
         <v>1</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="G41" s="1" t="n">
         <v>1</v>
@@ -6595,7 +6600,7 @@
     </row>
     <row r="42" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>1</v>
@@ -6610,7 +6615,7 @@
         <v>1</v>
       </c>
       <c r="F42" s="17" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="G42" s="1" t="n">
         <v>1</v>
@@ -6627,7 +6632,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>1</v>
@@ -6642,7 +6647,7 @@
         <v>1</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G43" s="1" t="n">
         <v>1</v>
@@ -6659,7 +6664,7 @@
     </row>
     <row r="44" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="17" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>1</v>
@@ -6674,7 +6679,7 @@
         <v>1</v>
       </c>
       <c r="F44" s="17" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G44" s="1" t="n">
         <v>1</v>
@@ -6691,7 +6696,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="17" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>1</v>
@@ -6706,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="F45" s="17" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G45" s="1" t="n">
         <v>1</v>
@@ -6793,18 +6798,8 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B13:E45">
+  <conditionalFormatting sqref="B13:E45 B2:E45 G2:J45">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:E45">
-    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:J45">
-    <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>